<commit_message>
TOTAL RH: set columns B-Q to 61 px wide
Uniform width (8.0 chars at Calibri 11) per user request,
overriding the earlier per-section widths.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_10-5.xlsx
+++ b/Stock_Daily_Reefer_10-5.xlsx
@@ -4389,7 +4389,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -4397,13 +4397,14 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">

</xml_diff>